<commit_message>
Se actualiza el formato en donde queda consolidada la informacion
</commit_message>
<xml_diff>
--- a/public/formato-examen version 2.xlsx
+++ b/public/formato-examen version 2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cristian\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cristian\Documents\SYP\Proyetos automatizacion 2\HL\Examenes medicos\web\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DA9D611-DBF8-47C3-ADDE-18F54F719DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58BF8F2F-E9B4-4762-AE7E-0550B3F108E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -551,14 +551,13 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -652,29 +651,76 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -714,55 +760,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -875,6 +873,10 @@
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
 </file>
 
+<file path=xl/ctrlProps/ctrlProp30.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+</file>
+
 <file path=xl/ctrlProps/ctrlProp4.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
 </file>
@@ -1594,15 +1596,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>45720</xdr:colOff>
+          <xdr:colOff>38100</xdr:colOff>
           <xdr:row>39</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
+          <xdr:rowOff>45720</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>9</xdr:col>
-          <xdr:colOff>1066800</xdr:colOff>
+          <xdr:colOff>1059180</xdr:colOff>
           <xdr:row>40</xdr:row>
-          <xdr:rowOff>7620</xdr:rowOff>
+          <xdr:rowOff>53340</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1680,15 +1682,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>45720</xdr:colOff>
+          <xdr:colOff>38100</xdr:colOff>
           <xdr:row>40</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:rowOff>60960</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>9</xdr:col>
-          <xdr:colOff>251460</xdr:colOff>
+          <xdr:colOff>243840</xdr:colOff>
           <xdr:row>41</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:rowOff>60960</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2375,8 +2377,8 @@
         <xdr:to>
           <xdr:col>9</xdr:col>
           <xdr:colOff>251460</xdr:colOff>
-          <xdr:row>35</xdr:row>
-          <xdr:rowOff>213360</xdr:rowOff>
+          <xdr:row>36</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2461,8 +2463,8 @@
         <xdr:to>
           <xdr:col>9</xdr:col>
           <xdr:colOff>952500</xdr:colOff>
-          <xdr:row>37</xdr:row>
-          <xdr:rowOff>213360</xdr:rowOff>
+          <xdr:row>38</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2547,8 +2549,8 @@
         <xdr:to>
           <xdr:col>9</xdr:col>
           <xdr:colOff>1028700</xdr:colOff>
-          <xdr:row>36</xdr:row>
-          <xdr:rowOff>213360</xdr:rowOff>
+          <xdr:row>37</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2628,13 +2630,13 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>30480</xdr:colOff>
           <xdr:row>42</xdr:row>
-          <xdr:rowOff>83820</xdr:rowOff>
+          <xdr:rowOff>30480</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>9</xdr:col>
           <xdr:colOff>1021080</xdr:colOff>
           <xdr:row>43</xdr:row>
-          <xdr:rowOff>160020</xdr:rowOff>
+          <xdr:rowOff>106680</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2714,13 +2716,13 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>30480</xdr:colOff>
           <xdr:row>43</xdr:row>
-          <xdr:rowOff>152400</xdr:rowOff>
+          <xdr:rowOff>83820</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>9</xdr:col>
           <xdr:colOff>228600</xdr:colOff>
           <xdr:row>44</xdr:row>
-          <xdr:rowOff>152400</xdr:rowOff>
+          <xdr:rowOff>83820</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2886,13 +2888,13 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>30480</xdr:colOff>
           <xdr:row>44</xdr:row>
-          <xdr:rowOff>144780</xdr:rowOff>
+          <xdr:rowOff>106680</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>9</xdr:col>
           <xdr:colOff>228600</xdr:colOff>
           <xdr:row>45</xdr:row>
-          <xdr:rowOff>144780</xdr:rowOff>
+          <xdr:rowOff>106680</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2970,15 +2972,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>45720</xdr:colOff>
+          <xdr:colOff>38100</xdr:colOff>
           <xdr:row>45</xdr:row>
-          <xdr:rowOff>182880</xdr:rowOff>
+          <xdr:rowOff>121920</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>9</xdr:col>
-          <xdr:colOff>251460</xdr:colOff>
-          <xdr:row>47</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
+          <xdr:colOff>243840</xdr:colOff>
+          <xdr:row>46</xdr:row>
+          <xdr:rowOff>129540</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3228,15 +3230,15 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>60960</xdr:colOff>
-          <xdr:row>37</xdr:row>
-          <xdr:rowOff>213360</xdr:rowOff>
+          <xdr:colOff>45720</xdr:colOff>
+          <xdr:row>38</xdr:row>
+          <xdr:rowOff>22860</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>9</xdr:col>
-          <xdr:colOff>502920</xdr:colOff>
+          <xdr:colOff>487680</xdr:colOff>
           <xdr:row>39</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:rowOff>60960</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3314,13 +3316,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>83820</xdr:colOff>
+          <xdr:colOff>114300</xdr:colOff>
           <xdr:row>46</xdr:row>
           <xdr:rowOff>22860</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
-          <xdr:colOff>373380</xdr:colOff>
+          <xdr:colOff>403860</xdr:colOff>
           <xdr:row>47</xdr:row>
           <xdr:rowOff>76200</xdr:rowOff>
         </xdr:to>
@@ -3444,6 +3446,92 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>5</xdr:col>
+          <xdr:colOff>30480</xdr:colOff>
+          <xdr:row>46</xdr:row>
+          <xdr:rowOff>152400</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>7</xdr:col>
+          <xdr:colOff>167640</xdr:colOff>
+          <xdr:row>48</xdr:row>
+          <xdr:rowOff>15240</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1058" name="Check Box 34" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1058"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9578E53-BD46-4FBE-738F-C3EBA6DBF60B}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:solidFill>
+                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
+                  </a:solidFill>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="27432" rIns="0" bIns="27432" anchor="ctr" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="l" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="es-CO" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Segoe UI"/>
+                  <a:cs typeface="Segoe UI"/>
+                </a:rPr>
+                <a:t>OTRO</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
 </xdr:wsDr>
 </file>
 
@@ -3755,59 +3843,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="78" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:13" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="78"/>
-      <c r="F3" s="78"/>
-      <c r="G3" s="78"/>
-      <c r="H3" s="78"/>
-      <c r="I3" s="78"/>
-      <c r="J3" s="78"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
       <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:13" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="62" t="s">
+      <c r="A5" s="65" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="63"/>
-      <c r="C5" s="63"/>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
-      <c r="J5" s="63"/>
-      <c r="K5" s="63"/>
-      <c r="L5" s="64"/>
+      <c r="B5" s="66"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="66"/>
+      <c r="I5" s="66"/>
+      <c r="J5" s="66"/>
+      <c r="K5" s="66"/>
+      <c r="L5" s="67"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C6" s="3"/>
@@ -3816,101 +3904,101 @@
       <c r="C7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="90" t="s">
+      <c r="D7" s="73" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="92"/>
-      <c r="F7" s="91"/>
-      <c r="H7" s="5" t="s">
+      <c r="E7" s="75"/>
+      <c r="F7" s="74"/>
+      <c r="H7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="56" t="s">
+      <c r="I7" s="73" t="s">
         <v>36</v>
       </c>
+      <c r="J7" s="74"/>
     </row>
     <row r="8" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="85"/>
-      <c r="E8" s="86"/>
-      <c r="F8" s="87"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="69"/>
+      <c r="F8" s="70"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
     </row>
     <row r="9" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="88">
+      <c r="D9" s="71">
         <v>20136</v>
       </c>
-      <c r="E9" s="89"/>
+      <c r="E9" s="72"/>
       <c r="H9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="I9" s="90" t="s">
+      <c r="I9" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="J9" s="91"/>
-      <c r="K9" s="6"/>
+      <c r="J9" s="74"/>
+      <c r="K9" s="5"/>
     </row>
     <row r="10" spans="1:13" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:13" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="62" t="s">
+      <c r="A11" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
-      <c r="G11" s="63"/>
-      <c r="H11" s="63"/>
-      <c r="I11" s="63"/>
-      <c r="J11" s="63"/>
-      <c r="K11" s="63"/>
-      <c r="L11" s="64"/>
+      <c r="B11" s="66"/>
+      <c r="C11" s="66"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="66"/>
+      <c r="F11" s="66"/>
+      <c r="G11" s="66"/>
+      <c r="H11" s="66"/>
+      <c r="I11" s="66"/>
+      <c r="J11" s="66"/>
+      <c r="K11" s="66"/>
+      <c r="L11" s="67"/>
     </row>
     <row r="12" spans="1:13" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="8"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="10"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="9"/>
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="8"/>
-      <c r="C13" s="11" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="59" t="s">
+      <c r="D13" s="77" t="s">
         <v>41</v>
       </c>
-      <c r="E13" s="59"/>
-      <c r="F13" s="59"/>
-      <c r="G13" s="59"/>
-      <c r="H13" s="59"/>
-      <c r="I13" s="59"/>
-      <c r="J13" s="59"/>
-      <c r="K13" s="10"/>
-      <c r="M13" s="12"/>
+      <c r="E13" s="77"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="77"/>
+      <c r="H13" s="77"/>
+      <c r="I13" s="77"/>
+      <c r="J13" s="77"/>
+      <c r="K13" s="9"/>
+      <c r="M13" s="11"/>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="8"/>
-      <c r="C14" s="11" t="s">
+      <c r="B14" s="7"/>
+      <c r="C14" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D14" s="60">
+      <c r="D14" s="78">
         <v>8800751</v>
       </c>
       <c r="E14" s="61"/>
@@ -3919,116 +4007,116 @@
       <c r="H14" s="61"/>
       <c r="I14" s="61"/>
       <c r="J14" s="61"/>
-      <c r="K14" s="13"/>
-      <c r="M14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="M14" s="11"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B15" s="8"/>
-      <c r="C15" s="11" t="s">
+      <c r="B15" s="7"/>
+      <c r="C15" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D15" s="68" t="s">
+      <c r="D15" s="82" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="69"/>
-      <c r="F15" s="69"/>
-      <c r="G15" s="69"/>
-      <c r="H15" s="69"/>
-      <c r="I15" s="69"/>
-      <c r="J15" s="69"/>
-      <c r="K15" s="13"/>
-      <c r="M15" s="14"/>
+      <c r="E15" s="83"/>
+      <c r="F15" s="83"/>
+      <c r="G15" s="83"/>
+      <c r="H15" s="83"/>
+      <c r="I15" s="83"/>
+      <c r="J15" s="83"/>
+      <c r="K15" s="12"/>
+      <c r="M15" s="13"/>
     </row>
     <row r="16" spans="1:13" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="15"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="19"/>
-      <c r="M16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="18"/>
+      <c r="M16" s="13"/>
     </row>
     <row r="17" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C17" s="3"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="M17" s="14"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="M17" s="13"/>
     </row>
     <row r="18" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="62" t="s">
+      <c r="A18" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="63"/>
-      <c r="C18" s="63"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="63"/>
-      <c r="H18" s="63"/>
-      <c r="I18" s="63"/>
-      <c r="J18" s="63"/>
-      <c r="K18" s="63"/>
-      <c r="L18" s="64"/>
-      <c r="M18" s="14"/>
+      <c r="B18" s="66"/>
+      <c r="C18" s="66"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
+      <c r="G18" s="66"/>
+      <c r="H18" s="66"/>
+      <c r="I18" s="66"/>
+      <c r="J18" s="66"/>
+      <c r="K18" s="66"/>
+      <c r="L18" s="67"/>
+      <c r="M18" s="13"/>
     </row>
     <row r="19" spans="1:15" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="21"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
-      <c r="K19" s="25"/>
-      <c r="M19" s="14"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="24"/>
+      <c r="M19" s="13"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B20" s="8"/>
-      <c r="C20" s="11" t="s">
+      <c r="B20" s="7"/>
+      <c r="C20" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="79"/>
-      <c r="E20" s="80"/>
-      <c r="F20" s="80"/>
-      <c r="G20" s="80"/>
-      <c r="H20" s="80"/>
-      <c r="I20" s="80"/>
-      <c r="J20" s="81"/>
-      <c r="K20" s="26"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="59"/>
+      <c r="G20" s="59"/>
+      <c r="H20" s="59"/>
+      <c r="I20" s="59"/>
+      <c r="J20" s="60"/>
+      <c r="K20" s="25"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B21" s="8"/>
-      <c r="C21" s="11" t="s">
+      <c r="B21" s="7"/>
+      <c r="C21" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="73" t="s">
+      <c r="D21" s="87" t="s">
         <v>40</v>
       </c>
-      <c r="E21" s="74"/>
-      <c r="F21" s="74"/>
-      <c r="G21" s="75"/>
-      <c r="H21" s="11" t="s">
+      <c r="E21" s="88"/>
+      <c r="F21" s="88"/>
+      <c r="G21" s="89"/>
+      <c r="H21" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="I21" s="76"/>
-      <c r="J21" s="77"/>
-      <c r="K21" s="13"/>
+      <c r="I21" s="90"/>
+      <c r="J21" s="91"/>
+      <c r="K21" s="12"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B22" s="8"/>
-      <c r="C22" s="11" t="s">
+      <c r="B22" s="7"/>
+      <c r="C22" s="10" t="s">
         <v>4</v>
       </c>
       <c r="D22" s="61"/>
@@ -4038,414 +4126,406 @@
       <c r="H22" s="61"/>
       <c r="I22" s="61"/>
       <c r="J22" s="61"/>
-      <c r="K22" s="13"/>
+      <c r="K22" s="12"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="8"/>
-      <c r="C23" s="11" t="s">
+      <c r="B23" s="7"/>
+      <c r="C23" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D23" s="84">
+      <c r="D23" s="64">
         <v>46217</v>
       </c>
-      <c r="E23" s="84"/>
-      <c r="F23" s="84"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="82" t="s">
+      <c r="E23" s="64"/>
+      <c r="F23" s="64"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="I23" s="83"/>
-      <c r="J23" s="28" t="s">
+      <c r="I23" s="63"/>
+      <c r="J23" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="K23" s="29"/>
+      <c r="K23" s="28"/>
     </row>
     <row r="24" spans="1:15" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="15"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="30"/>
-      <c r="J24" s="30"/>
-      <c r="K24" s="31"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="29"/>
+      <c r="I24" s="29"/>
+      <c r="J24" s="29"/>
+      <c r="K24" s="30"/>
     </row>
     <row r="25" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="62" t="s">
+      <c r="A26" s="65" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="63"/>
-      <c r="C26" s="63"/>
-      <c r="D26" s="63"/>
-      <c r="E26" s="63"/>
-      <c r="F26" s="63"/>
-      <c r="G26" s="63"/>
-      <c r="H26" s="63"/>
-      <c r="I26" s="63"/>
-      <c r="J26" s="63"/>
-      <c r="K26" s="63"/>
-      <c r="L26" s="64"/>
+      <c r="B26" s="66"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
+      <c r="F26" s="66"/>
+      <c r="G26" s="66"/>
+      <c r="H26" s="66"/>
+      <c r="I26" s="66"/>
+      <c r="J26" s="66"/>
+      <c r="K26" s="66"/>
+      <c r="L26" s="67"/>
     </row>
     <row r="27" spans="1:15" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="21"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="33"/>
-      <c r="K27" s="34"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="33"/>
     </row>
     <row r="28" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="8"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="65"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="10"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="79"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="9"/>
       <c r="M28" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="8"/>
-      <c r="C29" s="35"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="35"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="65"/>
-      <c r="I29" s="9" t="s">
+      <c r="B29" s="7"/>
+      <c r="C29" s="34"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="79"/>
+      <c r="I29" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="J29" s="66"/>
-      <c r="K29" s="67"/>
+      <c r="J29" s="80"/>
+      <c r="K29" s="81"/>
     </row>
     <row r="30" spans="1:15" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="15"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="36"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="37"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="30"/>
-      <c r="K30" s="31"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="35"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="36"/>
+      <c r="I30" s="29"/>
+      <c r="J30" s="29"/>
+      <c r="K30" s="30"/>
     </row>
     <row r="31" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="9"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
       <c r="O31" s="3"/>
     </row>
     <row r="32" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="62" t="s">
+      <c r="A32" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="B32" s="63"/>
-      <c r="C32" s="63"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="63"/>
-      <c r="F32" s="63"/>
-      <c r="G32" s="63"/>
-      <c r="H32" s="63"/>
-      <c r="I32" s="63"/>
-      <c r="J32" s="63"/>
-      <c r="K32" s="63"/>
-      <c r="L32" s="64"/>
+      <c r="B32" s="66"/>
+      <c r="C32" s="66"/>
+      <c r="D32" s="66"/>
+      <c r="E32" s="66"/>
+      <c r="F32" s="66"/>
+      <c r="G32" s="66"/>
+      <c r="H32" s="66"/>
+      <c r="I32" s="66"/>
+      <c r="J32" s="66"/>
+      <c r="K32" s="66"/>
+      <c r="L32" s="67"/>
     </row>
     <row r="33" spans="2:15" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="21"/>
-      <c r="C33" s="33"/>
-      <c r="D33" s="33"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="33"/>
-      <c r="G33" s="33"/>
-      <c r="H33" s="33"/>
-      <c r="I33" s="33"/>
-      <c r="J33" s="33"/>
-      <c r="K33" s="34"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="33"/>
       <c r="O33" s="3"/>
     </row>
     <row r="34" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B34" s="38"/>
-      <c r="C34" s="70" t="s">
+      <c r="B34" s="37"/>
+      <c r="C34" s="84" t="s">
         <v>22</v>
       </c>
-      <c r="D34" s="70"/>
-      <c r="E34" s="70"/>
-      <c r="F34" s="70"/>
-      <c r="G34" s="70"/>
-      <c r="H34" s="70"/>
-      <c r="I34" s="70"/>
-      <c r="J34" s="70"/>
-      <c r="K34" s="71"/>
+      <c r="D34" s="84"/>
+      <c r="E34" s="84"/>
+      <c r="F34" s="84"/>
+      <c r="G34" s="84"/>
+      <c r="H34" s="84"/>
+      <c r="I34" s="84"/>
+      <c r="J34" s="84"/>
+      <c r="K34" s="85"/>
       <c r="O34" s="3"/>
     </row>
     <row r="35" spans="2:15" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="8"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
-      <c r="K35" s="10"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="9"/>
       <c r="O35" s="3"/>
     </row>
     <row r="36" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="38"/>
-      <c r="K36" s="39"/>
+      <c r="B36" s="37"/>
+      <c r="K36" s="38"/>
       <c r="O36" s="3"/>
     </row>
     <row r="37" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="38"/>
-      <c r="K37" s="39"/>
+      <c r="B37" s="37"/>
+      <c r="K37" s="38"/>
       <c r="O37" s="3"/>
     </row>
     <row r="38" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="38"/>
-      <c r="K38" s="39"/>
+      <c r="B38" s="37"/>
+      <c r="K38" s="38"/>
       <c r="O38" s="3"/>
     </row>
     <row r="39" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="38"/>
-      <c r="K39" s="39"/>
+      <c r="B39" s="37"/>
+      <c r="K39" s="38"/>
       <c r="O39" s="3"/>
     </row>
     <row r="40" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="38"/>
-      <c r="K40" s="39"/>
+      <c r="B40" s="37"/>
+      <c r="K40" s="38"/>
       <c r="O40" s="3"/>
     </row>
     <row r="41" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="38"/>
-      <c r="K41" s="39"/>
+      <c r="B41" s="37"/>
+      <c r="K41" s="38"/>
       <c r="O41" s="3"/>
     </row>
     <row r="42" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="38"/>
-      <c r="K42" s="39"/>
+      <c r="B42" s="37"/>
+      <c r="K42" s="38"/>
       <c r="O42" s="3"/>
     </row>
     <row r="43" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="38"/>
-      <c r="K43" s="39"/>
+      <c r="B43" s="37"/>
+      <c r="K43" s="38"/>
       <c r="O43" s="3"/>
     </row>
     <row r="44" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="38"/>
-      <c r="K44" s="39"/>
+      <c r="B44" s="37"/>
+      <c r="K44" s="38"/>
       <c r="O44" s="3"/>
     </row>
     <row r="45" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="38"/>
-      <c r="K45" s="39"/>
+      <c r="B45" s="37"/>
+      <c r="K45" s="38"/>
       <c r="O45" s="3"/>
     </row>
     <row r="46" spans="2:15" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="38"/>
-      <c r="K46" s="39"/>
+      <c r="B46" s="37"/>
+      <c r="K46" s="38"/>
       <c r="O46" s="3"/>
     </row>
     <row r="47" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B47" s="38"/>
-      <c r="K47" s="39"/>
+      <c r="B47" s="37"/>
+      <c r="K47" s="38"/>
       <c r="O47" s="3"/>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B48" s="38"/>
-      <c r="K48" s="39"/>
+      <c r="B48" s="37"/>
+      <c r="H48" s="92"/>
+      <c r="I48" s="92"/>
+      <c r="J48" s="92"/>
+      <c r="K48" s="38"/>
       <c r="O48" s="3"/>
     </row>
     <row r="49" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="38"/>
-      <c r="C49" s="40" t="s">
+      <c r="B49" s="37"/>
+      <c r="C49" s="39" t="s">
         <v>23</v>
       </c>
       <c r="F49" s="3"/>
-      <c r="K49" s="39"/>
+      <c r="K49" s="38"/>
       <c r="O49" s="3"/>
     </row>
     <row r="50" spans="1:15" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="38"/>
-      <c r="C50" s="40"/>
-      <c r="K50" s="39"/>
+      <c r="B50" s="37"/>
+      <c r="C50" s="39"/>
+      <c r="K50" s="38"/>
       <c r="O50" s="3"/>
     </row>
     <row r="51" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="38"/>
-      <c r="C51" s="9" t="s">
+      <c r="B51" s="37"/>
+      <c r="C51" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D51" s="41"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="41"/>
-      <c r="G51" s="11"/>
-      <c r="H51" s="9" t="s">
+      <c r="D51" s="40"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="I51" s="11"/>
-      <c r="J51" s="9"/>
-      <c r="K51" s="10"/>
+      <c r="I51" s="10"/>
+      <c r="J51" s="8"/>
+      <c r="K51" s="9"/>
     </row>
     <row r="52" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="38"/>
-      <c r="C52" s="9" t="s">
+      <c r="B52" s="37"/>
+      <c r="C52" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D52" s="93"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="94"/>
-      <c r="G52" s="11"/>
-      <c r="H52" s="9" t="s">
+      <c r="D52" s="55"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="48"/>
+      <c r="G52" s="10"/>
+      <c r="H52" s="8" t="s">
         <v>38</v>
       </c>
       <c r="I52" s="3"/>
-      <c r="K52" s="39"/>
+      <c r="K52" s="38"/>
     </row>
     <row r="53" spans="1:15" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="42"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="30"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="16"/>
-      <c r="H53" s="30"/>
-      <c r="I53" s="44"/>
-      <c r="J53" s="45"/>
-      <c r="K53" s="46"/>
+      <c r="B53" s="41"/>
+      <c r="C53" s="29"/>
+      <c r="D53" s="29"/>
+      <c r="E53" s="29"/>
+      <c r="F53" s="42"/>
+      <c r="G53" s="15"/>
+      <c r="H53" s="29"/>
+      <c r="I53" s="43"/>
+      <c r="J53" s="44"/>
+      <c r="K53" s="45"/>
     </row>
     <row r="54" spans="1:15" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="55" spans="1:15" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="62" t="s">
+      <c r="A55" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="B55" s="72"/>
-      <c r="C55" s="72"/>
-      <c r="D55" s="72"/>
-      <c r="E55" s="72"/>
-      <c r="F55" s="72"/>
-      <c r="G55" s="72"/>
-      <c r="H55" s="72"/>
-      <c r="I55" s="72"/>
-      <c r="J55" s="72"/>
-      <c r="K55" s="72"/>
-      <c r="L55" s="64"/>
+      <c r="B55" s="86"/>
+      <c r="C55" s="86"/>
+      <c r="D55" s="86"/>
+      <c r="E55" s="86"/>
+      <c r="F55" s="86"/>
+      <c r="G55" s="86"/>
+      <c r="H55" s="86"/>
+      <c r="I55" s="86"/>
+      <c r="J55" s="86"/>
+      <c r="K55" s="86"/>
+      <c r="L55" s="67"/>
     </row>
     <row r="56" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="47"/>
-      <c r="C56" s="48" t="s">
+      <c r="B56" s="46"/>
+      <c r="C56" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="D56" s="48"/>
-      <c r="E56" s="48"/>
-      <c r="F56" s="48"/>
-      <c r="G56" s="48"/>
-      <c r="H56" s="48"/>
-      <c r="I56" s="49" t="s">
+      <c r="D56" s="47"/>
+      <c r="E56" s="47"/>
+      <c r="F56" s="47"/>
+      <c r="G56" s="47"/>
+      <c r="H56" s="47"/>
+      <c r="I56" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="J56" s="48"/>
-      <c r="K56" s="50"/>
+      <c r="J56" s="47"/>
+      <c r="K56" s="49"/>
     </row>
     <row r="57" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="38"/>
+      <c r="B57" s="37"/>
       <c r="C57" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I57" s="51"/>
-      <c r="K57" s="39"/>
+      <c r="I57" s="50"/>
+      <c r="K57" s="38"/>
     </row>
     <row r="58" spans="1:15" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="38"/>
+      <c r="B58" s="37"/>
       <c r="C58" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="I58" s="51"/>
-      <c r="K58" s="39"/>
+      <c r="I58" s="50"/>
+      <c r="K58" s="38"/>
     </row>
     <row r="59" spans="1:15" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="52"/>
-      <c r="C59" s="45"/>
-      <c r="D59" s="45"/>
-      <c r="E59" s="45"/>
-      <c r="F59" s="45"/>
-      <c r="G59" s="45"/>
-      <c r="H59" s="45"/>
-      <c r="I59" s="53"/>
-      <c r="J59" s="45"/>
-      <c r="K59" s="46"/>
+      <c r="B59" s="51"/>
+      <c r="C59" s="44"/>
+      <c r="D59" s="44"/>
+      <c r="E59" s="44"/>
+      <c r="F59" s="44"/>
+      <c r="G59" s="44"/>
+      <c r="H59" s="44"/>
+      <c r="I59" s="52"/>
+      <c r="J59" s="44"/>
+      <c r="K59" s="45"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C61" s="40" t="s">
+      <c r="C61" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="E61" s="57" t="s">
+      <c r="E61" s="76" t="s">
         <v>37</v>
       </c>
-      <c r="F61" s="57"/>
-      <c r="G61" s="57"/>
-      <c r="H61" s="57"/>
-      <c r="I61" s="57"/>
-      <c r="J61" s="57"/>
-      <c r="K61" s="6"/>
+      <c r="F61" s="76"/>
+      <c r="G61" s="76"/>
+      <c r="H61" s="76"/>
+      <c r="I61" s="76"/>
+      <c r="J61" s="76"/>
+      <c r="K61" s="5"/>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C62" s="40" t="s">
+      <c r="C62" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="E62" s="58" t="s">
+      <c r="E62" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="F62" s="58"/>
-      <c r="G62" s="58"/>
-      <c r="H62" s="58"/>
-      <c r="I62" s="58"/>
-      <c r="J62" s="58"/>
-      <c r="K62" s="6"/>
+      <c r="F62" s="57"/>
+      <c r="G62" s="57"/>
+      <c r="H62" s="57"/>
+      <c r="I62" s="57"/>
+      <c r="J62" s="57"/>
+      <c r="K62" s="5"/>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C64" s="54"/>
+      <c r="C64" s="53"/>
     </row>
     <row r="65" spans="3:11" x14ac:dyDescent="0.25">
-      <c r="C65" s="55"/>
+      <c r="C65" s="54"/>
       <c r="H65" s="3"/>
       <c r="J65" s="3"/>
       <c r="K65" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="E1:J3"/>
-    <mergeCell ref="B1:D3"/>
-    <mergeCell ref="D20:J20"/>
-    <mergeCell ref="D22:J22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="A5:L5"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="D7:F7"/>
+  <mergeCells count="28">
     <mergeCell ref="E61:J61"/>
     <mergeCell ref="E62:J62"/>
     <mergeCell ref="D13:J13"/>
@@ -4461,6 +4541,19 @@
     <mergeCell ref="D21:G21"/>
     <mergeCell ref="I21:J21"/>
     <mergeCell ref="A26:L26"/>
+    <mergeCell ref="H48:J48"/>
+    <mergeCell ref="E1:J3"/>
+    <mergeCell ref="B1:D3"/>
+    <mergeCell ref="D20:J20"/>
+    <mergeCell ref="D22:J22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="I7:J7"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.55118110236220474" bottom="0.55118110236220474" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="90" orientation="portrait" horizontalDpi="4294967293" verticalDpi="200" r:id="rId1"/>
@@ -4652,15 +4745,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>45720</xdr:colOff>
+                    <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>39</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
+                    <xdr:rowOff>45720</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>9</xdr:col>
-                    <xdr:colOff>1066800</xdr:colOff>
+                    <xdr:colOff>1059180</xdr:colOff>
                     <xdr:row>40</xdr:row>
-                    <xdr:rowOff>7620</xdr:rowOff>
+                    <xdr:rowOff>53340</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4674,15 +4767,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>45720</xdr:colOff>
+                    <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>40</xdr:row>
-                    <xdr:rowOff>38100</xdr:rowOff>
+                    <xdr:rowOff>60960</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>9</xdr:col>
-                    <xdr:colOff>251460</xdr:colOff>
+                    <xdr:colOff>243840</xdr:colOff>
                     <xdr:row>41</xdr:row>
-                    <xdr:rowOff>38100</xdr:rowOff>
+                    <xdr:rowOff>60960</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4918,13 +5011,13 @@
                     <xdr:col>5</xdr:col>
                     <xdr:colOff>30480</xdr:colOff>
                     <xdr:row>42</xdr:row>
-                    <xdr:rowOff>83820</xdr:rowOff>
+                    <xdr:rowOff>30480</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>9</xdr:col>
                     <xdr:colOff>1021080</xdr:colOff>
                     <xdr:row>43</xdr:row>
-                    <xdr:rowOff>160020</xdr:rowOff>
+                    <xdr:rowOff>106680</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4940,13 +5033,13 @@
                     <xdr:col>5</xdr:col>
                     <xdr:colOff>30480</xdr:colOff>
                     <xdr:row>43</xdr:row>
-                    <xdr:rowOff>152400</xdr:rowOff>
+                    <xdr:rowOff>83820</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>9</xdr:col>
                     <xdr:colOff>228600</xdr:colOff>
                     <xdr:row>44</xdr:row>
-                    <xdr:rowOff>152400</xdr:rowOff>
+                    <xdr:rowOff>83820</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4984,13 +5077,13 @@
                     <xdr:col>5</xdr:col>
                     <xdr:colOff>30480</xdr:colOff>
                     <xdr:row>44</xdr:row>
-                    <xdr:rowOff>144780</xdr:rowOff>
+                    <xdr:rowOff>106680</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>9</xdr:col>
                     <xdr:colOff>228600</xdr:colOff>
                     <xdr:row>45</xdr:row>
-                    <xdr:rowOff>144780</xdr:rowOff>
+                    <xdr:rowOff>106680</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -5004,15 +5097,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>45720</xdr:colOff>
+                    <xdr:colOff>38100</xdr:colOff>
                     <xdr:row>45</xdr:row>
-                    <xdr:rowOff>182880</xdr:rowOff>
+                    <xdr:rowOff>121920</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>9</xdr:col>
-                    <xdr:colOff>251460</xdr:colOff>
-                    <xdr:row>47</xdr:row>
-                    <xdr:rowOff>22860</xdr:rowOff>
+                    <xdr:colOff>243840</xdr:colOff>
+                    <xdr:row>46</xdr:row>
+                    <xdr:rowOff>129540</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -5070,15 +5163,15 @@
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>60960</xdr:colOff>
-                    <xdr:row>37</xdr:row>
-                    <xdr:rowOff>213360</xdr:rowOff>
+                    <xdr:colOff>45720</xdr:colOff>
+                    <xdr:row>38</xdr:row>
+                    <xdr:rowOff>22860</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>9</xdr:col>
-                    <xdr:colOff>502920</xdr:colOff>
+                    <xdr:colOff>487680</xdr:colOff>
                     <xdr:row>39</xdr:row>
-                    <xdr:rowOff>38100</xdr:rowOff>
+                    <xdr:rowOff>60960</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -5092,15 +5185,37 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>83820</xdr:colOff>
+                    <xdr:colOff>114300</xdr:colOff>
                     <xdr:row>46</xdr:row>
                     <xdr:rowOff>22860</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
-                    <xdr:colOff>373380</xdr:colOff>
+                    <xdr:colOff>403860</xdr:colOff>
                     <xdr:row>47</xdr:row>
                     <xdr:rowOff>76200</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1058" r:id="rId33" name="Check Box 34">
+              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>5</xdr:col>
+                    <xdr:colOff>30480</xdr:colOff>
+                    <xdr:row>46</xdr:row>
+                    <xdr:rowOff>152400</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>7</xdr:col>
+                    <xdr:colOff>167640</xdr:colOff>
+                    <xdr:row>48</xdr:row>
+                    <xdr:rowOff>15240</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>

</xml_diff>